<commit_message>
updating results to kras only (article)
</commit_message>
<xml_diff>
--- a/Results/Statistics/analysis_summary.xlsx
+++ b/Results/Statistics/analysis_summary.xlsx
@@ -477,19 +477,19 @@
         <v>12</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9600666666666646</v>
+        <v>0.09166666666666612</v>
       </c>
       <c r="E2" t="n">
-        <v>5.037450000000001</v>
+        <v>0.7333333333333331</v>
       </c>
       <c r="F2" t="n">
-        <v>1.895349999999993</v>
+        <v>0.4999999999999991</v>
       </c>
       <c r="G2" t="n">
-        <v>5.951594268623313</v>
+        <v>0.8519654162127326</v>
       </c>
       <c r="H2" t="n">
-        <v>16.72669999999999</v>
+        <v>1.5</v>
       </c>
     </row>
   </sheetData>
@@ -546,7 +546,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sotorasib</t>
+          <t>Adagrasib</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -556,22 +556,22 @@
         <v>12</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2046972222222182</v>
+        <v>-0.5250000000000004</v>
       </c>
       <c r="E2" t="n">
-        <v>5.186258333333334</v>
+        <v>0.7583333333333333</v>
       </c>
       <c r="F2" t="n">
-        <v>6.552393767797978</v>
+        <v>0.815694270457469</v>
       </c>
       <c r="G2" t="n">
-        <v>16.72669999999999</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Adagrasib</t>
+          <t>Daraxonrasib</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -581,16 +581,16 @@
         <v>12</v>
       </c>
       <c r="D3" t="n">
-        <v>1.715436111111111</v>
+        <v>0.7083333333333326</v>
       </c>
       <c r="E3" t="n">
-        <v>4.888641666666667</v>
+        <v>0.7083333333333326</v>
       </c>
       <c r="F3" t="n">
-        <v>5.267575910641726</v>
+        <v>0.1574347937582868</v>
       </c>
       <c r="G3" t="n">
-        <v>9.678799999999995</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -652,23 +652,23 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>KRAS-G13V</t>
+          <t>KRAS-G12R</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>2.461883333333333</v>
+        <v>-0.4000000000000004</v>
       </c>
       <c r="E2" t="n">
-        <v>6.90025</v>
+        <v>1.1</v>
       </c>
       <c r="F2" t="n">
-        <v>8.76201861934033</v>
+        <v>1.204989626511365</v>
       </c>
       <c r="G2" t="n">
-        <v>16.72669999999999</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="3">
@@ -679,23 +679,23 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>KRAS-G13C</t>
+          <t>KRAS-G12D</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>1.014116666666664</v>
+        <v>-0.4000000000000004</v>
       </c>
       <c r="E3" t="n">
-        <v>6.756416666666664</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>8.299739517217793</v>
+        <v>1.095445115010332</v>
       </c>
       <c r="G3" t="n">
-        <v>11.5346</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="4">
@@ -706,23 +706,23 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>KRAS-G12R</t>
+          <t>KRAS-G12V</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>-1.350016666666666</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="E4" t="n">
-        <v>5.638216666666669</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>6.155872256769686</v>
+        <v>1.095445115010332</v>
       </c>
       <c r="G4" t="n">
-        <v>7.621800000000007</v>
+        <v>1.300000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -733,23 +733,23 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>KRAS-G13A</t>
+          <t>KRAS-G12C</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.7398000000000025</v>
+        <v>-0.3500000000000005</v>
       </c>
       <c r="E5" t="n">
-        <v>5.62866666666667</v>
+        <v>0.9500000000000002</v>
       </c>
       <c r="F5" t="n">
-        <v>6.471485743474989</v>
+        <v>1.040672859259816</v>
       </c>
       <c r="G5" t="n">
-        <v>7.6387</v>
+        <v>1.300000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -760,23 +760,23 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>KRAS-G13D</t>
+          <t>KRAS-G13C</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>2.183583333333329</v>
+        <v>0.9499999999999993</v>
       </c>
       <c r="E6" t="n">
-        <v>5.34995</v>
+        <v>0.9499999999999993</v>
       </c>
       <c r="F6" t="n">
-        <v>5.996443439045071</v>
+        <v>0.2738612787525831</v>
       </c>
       <c r="G6" t="n">
-        <v>7.982699999999994</v>
+        <v>1.199999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -787,23 +787,23 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KRAS-G12V</t>
+          <t>KRAS-G12A</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>3.333349999999998</v>
+        <v>-0.4500000000000011</v>
       </c>
       <c r="E7" t="n">
-        <v>5.249416666666669</v>
+        <v>0.8499999999999996</v>
       </c>
       <c r="F7" t="n">
-        <v>6.096425477195633</v>
+        <v>0.9311283477587821</v>
       </c>
       <c r="G7" t="n">
-        <v>11.0739</v>
+        <v>1.300000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -821,16 +821,16 @@
         <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>1.640616666666663</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="E8" t="n">
-        <v>5.104883333333333</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="F8" t="n">
-        <v>6.998416538451155</v>
+        <v>0.7668115805072319</v>
       </c>
       <c r="G8" t="n">
-        <v>13.4079</v>
+        <v>0.8999999999999986</v>
       </c>
     </row>
     <row r="9">
@@ -841,23 +841,23 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>KRAS-G12S</t>
+          <t>KRAS-G13V</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>1.671266666666667</v>
+        <v>0.3999999999999999</v>
       </c>
       <c r="E9" t="n">
-        <v>4.269233333333331</v>
+        <v>0.6000000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>4.916791946245706</v>
+        <v>0.6572670690061995</v>
       </c>
       <c r="G9" t="n">
-        <v>7.879499999999993</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -868,23 +868,23 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KRAS-G12A</t>
+          <t>KRAS-G13R</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>3.909866666666665</v>
+        <v>0.3499999999999992</v>
       </c>
       <c r="E10" t="n">
-        <v>4.246433333333335</v>
+        <v>0.5499999999999994</v>
       </c>
       <c r="F10" t="n">
-        <v>3.257745471129796</v>
+        <v>0.602494813255682</v>
       </c>
       <c r="G10" t="n">
-        <v>8.440700000000007</v>
+        <v>0.8999999999999986</v>
       </c>
     </row>
     <row r="11">
@@ -895,23 +895,23 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>KRAS-G13R</t>
+          <t>KRAS-G12S</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>-1.526466666666669</v>
+        <v>0.3999999999999995</v>
       </c>
       <c r="E11" t="n">
-        <v>3.849000000000004</v>
+        <v>0.3999999999999995</v>
       </c>
       <c r="F11" t="n">
-        <v>5.117380891302376</v>
+        <v>0.3286335345030995</v>
       </c>
       <c r="G11" t="n">
-        <v>8.731200000000001</v>
+        <v>0.6999999999999993</v>
       </c>
     </row>
     <row r="12">
@@ -922,23 +922,23 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>KRAS-G12D</t>
+          <t>KRAS-G13A</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>0.7914499999999975</v>
+        <v>0.3999999999999995</v>
       </c>
       <c r="E12" t="n">
-        <v>3.80298333333333</v>
+        <v>0.3999999999999995</v>
       </c>
       <c r="F12" t="n">
-        <v>4.827492117342086</v>
+        <v>0.3286335345030995</v>
       </c>
       <c r="G12" t="n">
-        <v>9.034599999999998</v>
+        <v>0.6999999999999993</v>
       </c>
     </row>
     <row r="13">
@@ -949,23 +949,23 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>KRAS-G12C</t>
+          <t>KRAS-G13D</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>-1.869050000000001</v>
+        <v>0.2999999999999998</v>
       </c>
       <c r="E13" t="n">
-        <v>3.65395</v>
+        <v>0.2999999999999998</v>
       </c>
       <c r="F13" t="n">
-        <v>4.622836527825744</v>
+        <v>0.3286335345030995</v>
       </c>
       <c r="G13" t="n">
-        <v>9.324799999999996</v>
+        <v>0.5999999999999996</v>
       </c>
     </row>
   </sheetData>
@@ -1002,14 +1002,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Weaker</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="C2" t="n">
-        <v>54.16666666666666</v>
+        <v>70.83333333333334</v>
       </c>
     </row>
     <row r="3">
@@ -1019,23 +1019,23 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>40.27777777777778</v>
+        <v>20.83333333333334</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Weaker</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C4" t="n">
-        <v>5.555555555555555</v>
+        <v>8.333333333333332</v>
       </c>
     </row>
   </sheetData>
@@ -1073,13 +1073,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -1087,13 +1087,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D3" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -1101,13 +1101,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -1176,25 +1176,25 @@
         <v>72</v>
       </c>
       <c r="C2" t="n">
-        <v>10.745689403688</v>
+        <v>8.710063943548347</v>
       </c>
       <c r="D2" t="n">
-        <v>9.933148931134598</v>
+        <v>9.44415619727493</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2353324883982923</v>
+        <v>0.2124076614616669</v>
       </c>
       <c r="F2" t="n">
-        <v>1.717700255314938</v>
+        <v>0.6931960140741523</v>
       </c>
       <c r="G2" t="n">
-        <v>9.821428774674306</v>
+        <v>1.567772570538591</v>
       </c>
       <c r="H2" t="n">
-        <v>21.5610989725898</v>
+        <v>14.86211740250359</v>
       </c>
       <c r="I2" t="n">
-        <v>29.47945393518381</v>
+        <v>30.54101830792372</v>
       </c>
     </row>
   </sheetData>
@@ -1235,10 +1235,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.001684173598167598</v>
+        <v>-0.01160407004015288</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9887976025590823</v>
+        <v>0.9229298805678773</v>
       </c>
     </row>
     <row r="3">
@@ -1248,10 +1248,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.01397330767075692</v>
+        <v>0.07088007130596617</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9072578711621112</v>
+        <v>0.5540808138441639</v>
       </c>
     </row>
   </sheetData>

</xml_diff>